<commit_message>
update: actualizar plantilla Excel del informe médico
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/templates/Plantilla informe medico.xlsx
+++ b/app/templates/Plantilla informe medico.xlsx
@@ -263,84 +263,88 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -427,9 +431,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>797400</xdr:colOff>
+      <xdr:colOff>797040</xdr:colOff>
       <xdr:row>42</xdr:row>
-      <xdr:rowOff>161280</xdr:rowOff>
+      <xdr:rowOff>160920</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -443,7 +447,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2449800" y="7255080"/>
-          <a:ext cx="792360" cy="664560"/>
+          <a:ext cx="792000" cy="664200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -470,9 +474,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>569160</xdr:colOff>
+      <xdr:colOff>568800</xdr:colOff>
       <xdr:row>43</xdr:row>
-      <xdr:rowOff>160560</xdr:rowOff>
+      <xdr:rowOff>160200</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -486,7 +490,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2413080" y="7270560"/>
-          <a:ext cx="848520" cy="671760"/>
+          <a:ext cx="848160" cy="671400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -682,330 +686,330 @@
   <dimension ref="B3:I47"/>
   <sheetFormatPr defaultColWidth="10.6015625" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="9.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="7.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="4.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="9.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="7.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="14.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="4.82"/>
   </cols>
   <sheetData>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="6"/>
+      <c r="C11" s="7"/>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7" t="s">
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="H12" s="7"/>
+      <c r="H12" s="8"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="7" t="s">
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8" t="s">
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="H15" s="8"/>
+      <c r="H15" s="9"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="9"/>
+      <c r="C18" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C20" s="6"/>
+      <c r="C20" s="7"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="12"/>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="11"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
+      <c r="B23" s="12"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6" t="s">
+      <c r="C24" s="7"/>
+      <c r="D24" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="E24" s="6"/>
+      <c r="E24" s="7"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6" t="s">
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
-      <c r="H26" s="6"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
+      <c r="H26" s="7"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
-      <c r="E27" s="6" t="s">
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="7"/>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="12" t="s">
+      <c r="B29" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C29" s="12"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="12"/>
-      <c r="F29" s="12"/>
-      <c r="G29" s="12"/>
-      <c r="H29" s="12"/>
-      <c r="I29" s="12"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="13"/>
+      <c r="G29" s="13"/>
+      <c r="H29" s="13"/>
+      <c r="I29" s="13"/>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="13"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="13"/>
-      <c r="G30" s="13"/>
-      <c r="H30" s="13"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="14"/>
+      <c r="H30" s="14"/>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="14" t="s">
+      <c r="B31" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14" t="s">
+      <c r="C31" s="15"/>
+      <c r="D31" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14" t="s">
+      <c r="E31" s="15"/>
+      <c r="F31" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="G31" s="14"/>
-      <c r="H31" s="15" t="s">
+      <c r="G31" s="15"/>
+      <c r="H31" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="I31" s="15"/>
+      <c r="I31" s="16"/>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="14" t="s">
+      <c r="B32" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="C32" s="14"/>
-      <c r="D32" s="16"/>
-      <c r="E32" s="16"/>
-      <c r="F32" s="16"/>
-      <c r="G32" s="16"/>
-      <c r="H32" s="16"/>
-      <c r="I32" s="16"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="17"/>
+      <c r="H32" s="17"/>
+      <c r="I32" s="17"/>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="14" t="s">
+      <c r="B33" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="C33" s="14"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="16"/>
-      <c r="G33" s="16"/>
-      <c r="H33" s="16"/>
-      <c r="I33" s="16"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="17"/>
+      <c r="H33" s="17"/>
+      <c r="I33" s="17"/>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="14" t="s">
+      <c r="B34" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="C34" s="14"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="16"/>
-      <c r="F34" s="16"/>
-      <c r="G34" s="16"/>
-      <c r="H34" s="16"/>
-      <c r="I34" s="16"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="17"/>
+      <c r="G34" s="17"/>
+      <c r="H34" s="17"/>
+      <c r="I34" s="17"/>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="14" t="s">
+      <c r="B35" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="C35" s="14"/>
-      <c r="D35" s="16"/>
-      <c r="E35" s="16"/>
-      <c r="F35" s="16"/>
-      <c r="G35" s="16"/>
-      <c r="H35" s="16"/>
-      <c r="I35" s="16"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="17"/>
+      <c r="F35" s="17"/>
+      <c r="G35" s="17"/>
+      <c r="H35" s="17"/>
+      <c r="I35" s="17"/>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="14" t="s">
+      <c r="B36" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="C36" s="14"/>
-      <c r="D36" s="16"/>
-      <c r="E36" s="16"/>
-      <c r="F36" s="16"/>
-      <c r="G36" s="16"/>
-      <c r="H36" s="16"/>
-      <c r="I36" s="16"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="17"/>
+      <c r="F36" s="17"/>
+      <c r="G36" s="17"/>
+      <c r="H36" s="17"/>
+      <c r="I36" s="17"/>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="17"/>
-      <c r="C37" s="17"/>
+      <c r="B37" s="18"/>
+      <c r="C37" s="18"/>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="8" t="s">
+      <c r="B38" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C38" s="8"/>
-      <c r="D38" s="8"/>
-      <c r="E38" s="8"/>
-      <c r="F38" s="8"/>
+      <c r="C38" s="9"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="9"/>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D39" s="8" t="s">
+      <c r="D39" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="E39" s="8"/>
-      <c r="F39" s="8"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="9"/>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="18"/>
-      <c r="C40" s="18"/>
-      <c r="D40" s="18"/>
-      <c r="E40" s="18"/>
+      <c r="B40" s="19"/>
+      <c r="C40" s="19"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="19"/>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B46" s="19"/>
-      <c r="C46" s="19"/>
-      <c r="D46" s="19"/>
-      <c r="E46" s="19"/>
-      <c r="F46" s="19"/>
-      <c r="G46" s="19"/>
-      <c r="H46" s="19"/>
+      <c r="B46" s="20"/>
+      <c r="C46" s="20"/>
+      <c r="D46" s="20"/>
+      <c r="E46" s="20"/>
+      <c r="F46" s="20"/>
+      <c r="G46" s="20"/>
+      <c r="H46" s="20"/>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B47" s="19"/>
-      <c r="C47" s="19"/>
-      <c r="D47" s="19"/>
-      <c r="E47" s="19"/>
-      <c r="F47" s="19"/>
-      <c r="G47" s="19"/>
-      <c r="H47" s="19"/>
+      <c r="B47" s="20"/>
+      <c r="C47" s="20"/>
+      <c r="D47" s="20"/>
+      <c r="E47" s="20"/>
+      <c r="F47" s="20"/>
+      <c r="G47" s="20"/>
+      <c r="H47" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="48">
@@ -1078,24 +1082,24 @@
   <sheetFormatPr defaultColWidth="10.6015625" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>